<commit_message>
enrich check_block semantic output
</commit_message>
<xml_diff>
--- a/contracts/ChainSwap/output_debug/storage.xlsx
+++ b/contracts/ChainSwap/output_debug/storage.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,25 +451,30 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>semantic_with_type</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>var_type</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>is_package</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>slot_Offset</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>describe</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>blockID</t>
         </is>
@@ -496,23 +501,28 @@
           <t>_creator</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="b">
-        <v>1</v>
-      </c>
-      <c r="G2" t="inlineStr">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>address _creator</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>bytes 0 to 19</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x69</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>0x573</t>
         </is>
@@ -539,23 +549,28 @@
           <t>_authQuotaOf</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G3" t="inlineStr">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>mapping (address =&gt; uint256) _authQuotaOf</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="b">
+        <v>0</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>bytes 0 to 31</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>🔵 Mapping (Datalog 跨块追踪)-&gt; Base Slot: 0x6a (0x5a7)</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>0x599</t>
         </is>
@@ -582,23 +597,28 @@
           <t>_mainChainId</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="b">
-        <v>0</v>
-      </c>
-      <c r="G4" t="inlineStr">
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>uint256 _mainChainId</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="b">
+        <v>0</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>bytes 0 to 31</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x67</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>0x5b1</t>
         </is>
@@ -625,23 +645,28 @@
           <t>_received</t>
         </is>
       </c>
-      <c r="E5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G5" t="inlineStr">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>mapping (uint256 =&gt; mapping (address =&gt; mapping (uint256 =&gt; uint256))) _received</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>bytes 0 to 31</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>🔵 Mapping (Datalog 跨块追踪)-&gt; Base Slot: 0x6d (0x6f9)</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>0x6d3</t>
         </is>
@@ -668,23 +693,28 @@
           <t>_sentCount</t>
         </is>
       </c>
-      <c r="E6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G6" t="inlineStr">
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>mapping (uint256 =&gt; mapping (address =&gt; uint256)) _sentCount</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>bytes 0 to 31</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>🔵 Mapping (Datalog 跨块追踪)-&gt; Base Slot: 0x6b (0x769)</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>0x719</t>
         </is>
@@ -711,23 +741,28 @@
           <t>_dOMAIN_SEPARATOR</t>
         </is>
       </c>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G7" t="inlineStr">
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>bytes32 _dOMAIN_SEPARATOR</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="b">
+        <v>0</v>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>bytes 0 to 31</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x65</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>0x850</t>
         </is>
@@ -754,23 +789,28 @@
           <t>_sent</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" t="b">
-        <v>0</v>
-      </c>
-      <c r="G8" t="inlineStr">
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>mapping (uint256 =&gt; mapping (address =&gt; mapping (uint256 =&gt; uint256))) _sent</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="b">
+        <v>0</v>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>bytes 0 to 31</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>🔵 Mapping (Datalog 跨块追踪)-&gt; Base Slot: 0x6c (0xa77)</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>0xa51</t>
         </is>
@@ -797,23 +837,28 @@
           <t>_received</t>
         </is>
       </c>
-      <c r="E9" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" t="b">
-        <v>0</v>
-      </c>
-      <c r="G9" t="inlineStr">
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>mapping (uint256 =&gt; mapping (address =&gt; mapping (uint256 =&gt; uint256))) _received</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="b">
+        <v>0</v>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>bytes 0 to 31</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>🔵 Mapping (Datalog 跨块追踪)-&gt; Base Slot: 0x6d (0xda8)</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>0xd45</t>
         </is>
@@ -840,23 +885,28 @@
           <t>_factory</t>
         </is>
       </c>
-      <c r="E10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" t="b">
-        <v>1</v>
-      </c>
-      <c r="G10" t="inlineStr">
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>address _factory</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>bytes 0 to 19</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x66</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>0xde9</t>
         </is>
@@ -883,23 +933,28 @@
           <t>_dOMAIN_SEPARATOR</t>
         </is>
       </c>
-      <c r="E11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" t="b">
-        <v>0</v>
-      </c>
-      <c r="G11" t="inlineStr">
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>bytes32 _dOMAIN_SEPARATOR</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="b">
+        <v>0</v>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>bytes 0 to 31</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x65</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>0x1011</t>
         </is>
@@ -926,23 +981,28 @@
           <t>___TokenMapped_init</t>
         </is>
       </c>
-      <c r="E12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" t="b">
-        <v>1</v>
-      </c>
-      <c r="G12" t="inlineStr">
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>bool ___TokenMapped_init</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="b">
+        <v>1</v>
+      </c>
+      <c r="H12" t="inlineStr">
         <is>
           <t>bytes 1 to 1</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x0</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>0x1348</t>
         </is>
@@ -969,23 +1029,28 @@
           <t>stor_0_0_0</t>
         </is>
       </c>
-      <c r="E13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" t="b">
-        <v>1</v>
-      </c>
-      <c r="G13" t="inlineStr">
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>bool stor_0_0_0</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="b">
+        <v>1</v>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>bytes 0 to 0</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x0</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>0x136d</t>
         </is>
@@ -1012,23 +1077,28 @@
           <t>___TokenMapped_init</t>
         </is>
       </c>
-      <c r="E14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" t="b">
-        <v>1</v>
-      </c>
-      <c r="G14" t="inlineStr">
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>bool ___TokenMapped_init</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="b">
+        <v>1</v>
+      </c>
+      <c r="H14" t="inlineStr">
         <is>
           <t>bytes 1 to 1</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x0</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>0x13bc</t>
         </is>
@@ -1055,23 +1125,28 @@
           <t>___TokenMapped_init</t>
         </is>
       </c>
-      <c r="E15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" t="b">
-        <v>1</v>
-      </c>
-      <c r="G15" t="inlineStr">
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>bool ___TokenMapped_init</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="b">
+        <v>1</v>
+      </c>
+      <c r="H15" t="inlineStr">
         <is>
           <t>bytes 1 to 1</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x0</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>0x13d7</t>
         </is>
@@ -1098,23 +1173,28 @@
           <t>stor_0_0_0</t>
         </is>
       </c>
-      <c r="E16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" t="b">
-        <v>1</v>
-      </c>
-      <c r="G16" t="inlineStr">
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>bool stor_0_0_0</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="b">
+        <v>1</v>
+      </c>
+      <c r="H16" t="inlineStr">
         <is>
           <t>bytes 0 to 0</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x0</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>0x13d7</t>
         </is>
@@ -1141,23 +1221,28 @@
           <t>_factory</t>
         </is>
       </c>
-      <c r="E17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" t="b">
-        <v>1</v>
-      </c>
-      <c r="G17" t="inlineStr">
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>address _factory</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="b">
+        <v>1</v>
+      </c>
+      <c r="H17" t="inlineStr">
         <is>
           <t>bytes 0 to 19</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x66</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>0x140c</t>
         </is>
@@ -1184,23 +1269,28 @@
           <t>_token</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" t="b">
-        <v>1</v>
-      </c>
-      <c r="G18" t="inlineStr">
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>address _token</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="b">
+        <v>1</v>
+      </c>
+      <c r="H18" t="inlineStr">
         <is>
           <t>bytes 0 to 19</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x68</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>0x1455</t>
         </is>
@@ -1227,23 +1317,28 @@
           <t>_creator</t>
         </is>
       </c>
-      <c r="E19" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" t="b">
-        <v>1</v>
-      </c>
-      <c r="G19" t="inlineStr">
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>address _creator</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="b">
+        <v>1</v>
+      </c>
+      <c r="H19" t="inlineStr">
         <is>
           <t>bytes 0 to 19</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x69</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>0x1455</t>
         </is>
@@ -1270,23 +1365,28 @@
           <t>_token</t>
         </is>
       </c>
-      <c r="E20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" t="b">
-        <v>1</v>
-      </c>
-      <c r="G20" t="inlineStr">
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>address _token</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="b">
+        <v>1</v>
+      </c>
+      <c r="H20" t="inlineStr">
         <is>
           <t>bytes 0 to 19</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x68</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>0x1455</t>
         </is>
@@ -1313,23 +1413,28 @@
           <t>___TokenMapped_init</t>
         </is>
       </c>
-      <c r="E21" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" t="b">
-        <v>1</v>
-      </c>
-      <c r="G21" t="inlineStr">
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>bool ___TokenMapped_init</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="b">
+        <v>1</v>
+      </c>
+      <c r="H21" t="inlineStr">
         <is>
           <t>bytes 1 to 1</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x0</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>0x15ea</t>
         </is>
@@ -1356,23 +1461,28 @@
           <t>_factory</t>
         </is>
       </c>
-      <c r="E22" t="n">
-        <v>0</v>
-      </c>
-      <c r="F22" t="b">
-        <v>1</v>
-      </c>
-      <c r="G22" t="inlineStr">
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>address _factory</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="b">
+        <v>1</v>
+      </c>
+      <c r="H22" t="inlineStr">
         <is>
           <t>bytes 0 to 19</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x66</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>0x1609</t>
         </is>
@@ -1399,23 +1509,28 @@
           <t>_token</t>
         </is>
       </c>
-      <c r="E23" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" t="b">
-        <v>1</v>
-      </c>
-      <c r="G23" t="inlineStr">
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>address _token</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="b">
+        <v>1</v>
+      </c>
+      <c r="H23" t="inlineStr">
         <is>
           <t>bytes 0 to 19</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x68</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>0x16e1</t>
         </is>
@@ -1442,23 +1557,28 @@
           <t>_sentCount</t>
         </is>
       </c>
-      <c r="E24" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" t="b">
-        <v>0</v>
-      </c>
-      <c r="G24" t="inlineStr">
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>mapping (uint256 =&gt; mapping (address =&gt; uint256)) _sentCount</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" t="b">
+        <v>0</v>
+      </c>
+      <c r="H24" t="inlineStr">
         <is>
           <t>bytes 0 to 31</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>🔵 Mapping (Datalog 跨块追踪)-&gt; Base Slot: 0x6b (0x1721)</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>0x1707</t>
         </is>
@@ -1485,23 +1605,28 @@
           <t>_factory</t>
         </is>
       </c>
-      <c r="E25" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" t="b">
-        <v>1</v>
-      </c>
-      <c r="G25" t="inlineStr">
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>address _factory</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="b">
+        <v>1</v>
+      </c>
+      <c r="H25" t="inlineStr">
         <is>
           <t>bytes 0 to 19</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x66</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>0x172c</t>
         </is>
@@ -1528,23 +1653,28 @@
           <t>_factory</t>
         </is>
       </c>
-      <c r="E26" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" t="b">
-        <v>1</v>
-      </c>
-      <c r="G26" t="inlineStr">
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>address _factory</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="b">
+        <v>1</v>
+      </c>
+      <c r="H26" t="inlineStr">
         <is>
           <t>bytes 0 to 19</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x66</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>0x1839</t>
         </is>
@@ -1571,23 +1701,28 @@
           <t>_factory</t>
         </is>
       </c>
-      <c r="E27" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" t="b">
-        <v>1</v>
-      </c>
-      <c r="G27" t="inlineStr">
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>address _factory</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="b">
+        <v>1</v>
+      </c>
+      <c r="H27" t="inlineStr">
         <is>
           <t>bytes 0 to 19</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x66</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="J27" t="inlineStr">
         <is>
           <t>0x193e</t>
         </is>
@@ -1614,23 +1749,28 @@
           <t>_token</t>
         </is>
       </c>
-      <c r="E28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" t="b">
-        <v>1</v>
-      </c>
-      <c r="G28" t="inlineStr">
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>address _token</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" t="b">
+        <v>1</v>
+      </c>
+      <c r="H28" t="inlineStr">
         <is>
           <t>bytes 0 to 19</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x68</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="J28" t="inlineStr">
         <is>
           <t>0x1a19</t>
         </is>
@@ -1657,23 +1797,28 @@
           <t>___TokenMapped_init</t>
         </is>
       </c>
-      <c r="E29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F29" t="b">
-        <v>1</v>
-      </c>
-      <c r="G29" t="inlineStr">
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>bool ___TokenMapped_init</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="b">
+        <v>1</v>
+      </c>
+      <c r="H29" t="inlineStr">
         <is>
           <t>bytes 1 to 1</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x0</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="J29" t="inlineStr">
         <is>
           <t>0x1a83</t>
         </is>
@@ -1700,23 +1845,28 @@
           <t>stor_0_0_0</t>
         </is>
       </c>
-      <c r="E30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" t="b">
-        <v>1</v>
-      </c>
-      <c r="G30" t="inlineStr">
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>bool stor_0_0_0</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="b">
+        <v>1</v>
+      </c>
+      <c r="H30" t="inlineStr">
         <is>
           <t>bytes 0 to 0</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x0</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="J30" t="inlineStr">
         <is>
           <t>0x1aa8</t>
         </is>
@@ -1743,23 +1893,28 @@
           <t>___TokenMapped_init</t>
         </is>
       </c>
-      <c r="E31" t="n">
-        <v>0</v>
-      </c>
-      <c r="F31" t="b">
-        <v>1</v>
-      </c>
-      <c r="G31" t="inlineStr">
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>bool ___TokenMapped_init</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="b">
+        <v>1</v>
+      </c>
+      <c r="H31" t="inlineStr">
         <is>
           <t>bytes 1 to 1</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x0</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="J31" t="inlineStr">
         <is>
           <t>0x1af7</t>
         </is>
@@ -1786,23 +1941,28 @@
           <t>___TokenMapped_init</t>
         </is>
       </c>
-      <c r="E32" t="n">
-        <v>0</v>
-      </c>
-      <c r="F32" t="b">
-        <v>1</v>
-      </c>
-      <c r="G32" t="inlineStr">
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>bool ___TokenMapped_init</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" t="b">
+        <v>1</v>
+      </c>
+      <c r="H32" t="inlineStr">
         <is>
           <t>bytes 1 to 1</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="I32" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x0</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="J32" t="inlineStr">
         <is>
           <t>0x1b12</t>
         </is>
@@ -1829,23 +1989,28 @@
           <t>stor_0_0_0</t>
         </is>
       </c>
-      <c r="E33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F33" t="b">
-        <v>1</v>
-      </c>
-      <c r="G33" t="inlineStr">
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>bool stor_0_0_0</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="b">
+        <v>1</v>
+      </c>
+      <c r="H33" t="inlineStr">
         <is>
           <t>bytes 0 to 0</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x0</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="J33" t="inlineStr">
         <is>
           <t>0x1b12</t>
         </is>
@@ -1872,23 +2037,28 @@
           <t>___TokenMapped_init</t>
         </is>
       </c>
-      <c r="E34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F34" t="b">
-        <v>1</v>
-      </c>
-      <c r="G34" t="inlineStr">
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>bool ___TokenMapped_init</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="b">
+        <v>1</v>
+      </c>
+      <c r="H34" t="inlineStr">
         <is>
           <t>bytes 1 to 1</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x0</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="J34" t="inlineStr">
         <is>
           <t>0x1b4e</t>
         </is>
@@ -1915,23 +2085,28 @@
           <t>_token</t>
         </is>
       </c>
-      <c r="E35" t="n">
-        <v>0</v>
-      </c>
-      <c r="F35" t="b">
-        <v>1</v>
-      </c>
-      <c r="G35" t="inlineStr">
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>address _token</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="b">
+        <v>1</v>
+      </c>
+      <c r="H35" t="inlineStr">
         <is>
           <t>bytes 0 to 19</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x68</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="J35" t="inlineStr">
         <is>
           <t>0x1cb8</t>
         </is>
@@ -1958,23 +2133,28 @@
           <t>_authQuotaOf</t>
         </is>
       </c>
-      <c r="E36" t="n">
-        <v>1</v>
-      </c>
-      <c r="F36" t="b">
-        <v>0</v>
-      </c>
-      <c r="G36" t="inlineStr">
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>mapping (address =&gt; uint256) _authQuotaOf</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" t="b">
+        <v>0</v>
+      </c>
+      <c r="H36" t="inlineStr">
         <is>
           <t>bytes 0 to 31</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>🔵 Mapping (Datalog 跨块追踪)-&gt; Base Slot: 0x6a (0x4700x1bb0)</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="J36" t="inlineStr">
         <is>
           <t>0x1b6b0x470</t>
         </is>
@@ -2001,23 +2181,28 @@
           <t>_authQuotaOf</t>
         </is>
       </c>
-      <c r="E37" t="n">
-        <v>1</v>
-      </c>
-      <c r="F37" t="b">
-        <v>0</v>
-      </c>
-      <c r="G37" t="inlineStr">
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>mapping (address =&gt; uint256) _authQuotaOf</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" t="b">
+        <v>0</v>
+      </c>
+      <c r="H37" t="inlineStr">
         <is>
           <t>bytes 0 to 31</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t>🔵 Mapping (Datalog 跨块追踪)-&gt; Base Slot: 0x6a (0x39b0xb58)</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="J37" t="inlineStr">
         <is>
           <t>0xb150x39b</t>
         </is>
@@ -2044,23 +2229,28 @@
           <t>_factory</t>
         </is>
       </c>
-      <c r="E38" t="n">
-        <v>0</v>
-      </c>
-      <c r="F38" t="b">
-        <v>1</v>
-      </c>
-      <c r="G38" t="inlineStr">
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>address _factory</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" t="b">
+        <v>1</v>
+      </c>
+      <c r="H38" t="inlineStr">
         <is>
           <t>bytes 0 to 19</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="I38" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x66</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="J38" t="inlineStr">
         <is>
           <t>0xa830x39b</t>
         </is>
@@ -2087,23 +2277,28 @@
           <t>_token</t>
         </is>
       </c>
-      <c r="E39" t="n">
-        <v>0</v>
-      </c>
-      <c r="F39" t="b">
-        <v>1</v>
-      </c>
-      <c r="G39" t="inlineStr">
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>address _token</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="b">
+        <v>1</v>
+      </c>
+      <c r="H39" t="inlineStr">
         <is>
           <t>bytes 0 to 19</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x68</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="J39" t="inlineStr">
         <is>
           <t>0x162fB0x4ec</t>
         </is>
@@ -2130,23 +2325,28 @@
           <t>___TokenMapped_init</t>
         </is>
       </c>
-      <c r="E40" t="n">
-        <v>0</v>
-      </c>
-      <c r="F40" t="b">
-        <v>1</v>
-      </c>
-      <c r="G40" t="inlineStr">
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>bool ___TokenMapped_init</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" t="b">
+        <v>1</v>
+      </c>
+      <c r="H40" t="inlineStr">
         <is>
           <t>bytes 1 to 1</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x0</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="J40" t="inlineStr">
         <is>
           <t>0x8e9B0x2ef</t>
         </is>
@@ -2173,23 +2373,28 @@
           <t>stor_0_0_0</t>
         </is>
       </c>
-      <c r="E41" t="n">
-        <v>0</v>
-      </c>
-      <c r="F41" t="b">
-        <v>1</v>
-      </c>
-      <c r="G41" t="inlineStr">
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>bool stor_0_0_0</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" t="b">
+        <v>1</v>
+      </c>
+      <c r="H41" t="inlineStr">
         <is>
           <t>bytes 0 to 0</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="I41" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x0</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="J41" t="inlineStr">
         <is>
           <t>0x8e9B0x2ef</t>
         </is>
@@ -2216,23 +2421,28 @@
           <t>___TokenMapped_init</t>
         </is>
       </c>
-      <c r="E42" t="n">
-        <v>0</v>
-      </c>
-      <c r="F42" t="b">
-        <v>1</v>
-      </c>
-      <c r="G42" t="inlineStr">
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>bool ___TokenMapped_init</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" t="b">
+        <v>1</v>
+      </c>
+      <c r="H42" t="inlineStr">
         <is>
           <t>bytes 1 to 1</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x0</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="J42" t="inlineStr">
         <is>
           <t>0x937B0x2ef</t>
         </is>
@@ -2259,23 +2469,28 @@
           <t>___TokenMapped_init</t>
         </is>
       </c>
-      <c r="E43" t="n">
-        <v>0</v>
-      </c>
-      <c r="F43" t="b">
-        <v>1</v>
-      </c>
-      <c r="G43" t="inlineStr">
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>bool ___TokenMapped_init</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" t="b">
+        <v>1</v>
+      </c>
+      <c r="H43" t="inlineStr">
         <is>
           <t>bytes 1 to 1</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x0</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="J43" t="inlineStr">
         <is>
           <t>0x85aB0x2ef</t>
         </is>
@@ -2302,23 +2517,28 @@
           <t>___TokenMapped_init</t>
         </is>
       </c>
-      <c r="E44" t="n">
-        <v>0</v>
-      </c>
-      <c r="F44" t="b">
-        <v>1</v>
-      </c>
-      <c r="G44" t="inlineStr">
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>bool ___TokenMapped_init</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" t="b">
+        <v>1</v>
+      </c>
+      <c r="H44" t="inlineStr">
         <is>
           <t>bytes 1 to 1</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="I44" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x0</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="J44" t="inlineStr">
         <is>
           <t>0x8ceB0x2ef</t>
         </is>
@@ -2345,23 +2565,28 @@
           <t>stor_0_0_0</t>
         </is>
       </c>
-      <c r="E45" t="n">
-        <v>0</v>
-      </c>
-      <c r="F45" t="b">
-        <v>1</v>
-      </c>
-      <c r="G45" t="inlineStr">
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>bool stor_0_0_0</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="b">
+        <v>1</v>
+      </c>
+      <c r="H45" t="inlineStr">
         <is>
           <t>bytes 0 to 0</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x0</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="J45" t="inlineStr">
         <is>
           <t>0x87fB0x2ef</t>
         </is>
@@ -2388,23 +2613,28 @@
           <t>_factory</t>
         </is>
       </c>
-      <c r="E46" t="n">
-        <v>0</v>
-      </c>
-      <c r="F46" t="b">
-        <v>1</v>
-      </c>
-      <c r="G46" t="inlineStr">
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>address _factory</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" t="b">
+        <v>1</v>
+      </c>
+      <c r="H46" t="inlineStr">
         <is>
           <t>bytes 0 to 19</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="I46" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x66</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="J46" t="inlineStr">
         <is>
           <t>0x95fB0x343</t>
         </is>
@@ -2431,23 +2661,28 @@
           <t>_authQuotaOf</t>
         </is>
       </c>
-      <c r="E47" t="n">
-        <v>1</v>
-      </c>
-      <c r="F47" t="b">
-        <v>0</v>
-      </c>
-      <c r="G47" t="inlineStr">
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>mapping (address =&gt; uint256) _authQuotaOf</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" t="b">
+        <v>0</v>
+      </c>
+      <c r="H47" t="inlineStr">
         <is>
           <t>bytes 0 to 31</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="I47" t="inlineStr">
         <is>
           <t>🔵 Mapping (Datalog 跨块追踪)-&gt; Base Slot: 0x6a (0x95f0x1bb0V0x343)</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
+      <c r="J47" t="inlineStr">
         <is>
           <t>0x1b6b0x95fB0x343</t>
         </is>
@@ -2474,23 +2709,28 @@
           <t>_authQuotaOf</t>
         </is>
       </c>
-      <c r="E48" t="n">
-        <v>1</v>
-      </c>
-      <c r="F48" t="b">
-        <v>0</v>
-      </c>
-      <c r="G48" t="inlineStr">
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>mapping (address =&gt; uint256) _authQuotaOf</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" t="b">
+        <v>0</v>
+      </c>
+      <c r="H48" t="inlineStr">
         <is>
           <t>bytes 0 to 31</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
+      <c r="I48" t="inlineStr">
         <is>
           <t>🔵 Mapping (Datalog 跨块追踪)-&gt; Base Slot: 0x6a (0x95f0xa30V0x343)</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr">
+      <c r="J48" t="inlineStr">
         <is>
           <t>0x9f10x95fB0x343</t>
         </is>
@@ -2517,23 +2757,28 @@
           <t>_authQuotaOf</t>
         </is>
       </c>
-      <c r="E49" t="n">
-        <v>1</v>
-      </c>
-      <c r="F49" t="b">
-        <v>0</v>
-      </c>
-      <c r="G49" t="inlineStr">
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>mapping (address =&gt; uint256) _authQuotaOf</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" t="b">
+        <v>0</v>
+      </c>
+      <c r="H49" t="inlineStr">
         <is>
           <t>bytes 0 to 31</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
+      <c r="I49" t="inlineStr">
         <is>
           <t>🔵 Mapping (Datalog 跨块追踪)-&gt; Base Slot: 0x6a (0x5b70xb58V0x1ef)</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
+      <c r="J49" t="inlineStr">
         <is>
           <t>0xb150x5b7B0x1ef</t>
         </is>
@@ -2560,23 +2805,28 @@
           <t>_factory</t>
         </is>
       </c>
-      <c r="E50" t="n">
-        <v>0</v>
-      </c>
-      <c r="F50" t="b">
-        <v>1</v>
-      </c>
-      <c r="G50" t="inlineStr">
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>address _factory</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" t="b">
+        <v>1</v>
+      </c>
+      <c r="H50" t="inlineStr">
         <is>
           <t>bytes 0 to 19</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr">
+      <c r="I50" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x66</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
+      <c r="J50" t="inlineStr">
         <is>
           <t>0xa830x5b7B0x1ef</t>
         </is>
@@ -2603,23 +2853,28 @@
           <t>_authQuotaOf</t>
         </is>
       </c>
-      <c r="E51" t="n">
-        <v>1</v>
-      </c>
-      <c r="F51" t="b">
-        <v>0</v>
-      </c>
-      <c r="G51" t="inlineStr">
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>mapping (address =&gt; uint256) _authQuotaOf</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" t="b">
+        <v>0</v>
+      </c>
+      <c r="H51" t="inlineStr">
         <is>
           <t>bytes 0 to 31</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr">
+      <c r="I51" t="inlineStr">
         <is>
           <t>🔵 Mapping (Datalog 跨块追踪)-&gt; Base Slot: 0x6a (0xc450x1bb0V0x455)</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr">
+      <c r="J51" t="inlineStr">
         <is>
           <t>0x1b6b0xc45B0x455</t>
         </is>
@@ -2646,23 +2901,28 @@
           <t>_authQuotaOf</t>
         </is>
       </c>
-      <c r="E52" t="n">
-        <v>1</v>
-      </c>
-      <c r="F52" t="b">
-        <v>0</v>
-      </c>
-      <c r="G52" t="inlineStr">
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>mapping (address =&gt; uint256) _authQuotaOf</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" t="b">
+        <v>0</v>
+      </c>
+      <c r="H52" t="inlineStr">
         <is>
           <t>bytes 0 to 31</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
+      <c r="I52" t="inlineStr">
         <is>
           <t>🔵 Mapping (Datalog 跨块追踪)-&gt; Base Slot: 0x6a (0xc450xa30V0x455)</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr">
+      <c r="J52" t="inlineStr">
         <is>
           <t>0x9f10xc45B0x455</t>
         </is>
@@ -2689,23 +2949,28 @@
           <t>_factory</t>
         </is>
       </c>
-      <c r="E53" t="n">
-        <v>0</v>
-      </c>
-      <c r="F53" t="b">
-        <v>1</v>
-      </c>
-      <c r="G53" t="inlineStr">
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>address _factory</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" t="b">
+        <v>1</v>
+      </c>
+      <c r="H53" t="inlineStr">
         <is>
           <t>bytes 0 to 19</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
+      <c r="I53" t="inlineStr">
         <is>
           <t>🟢 普通变量 (Normal)-&gt; Slot: 0x66</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr">
+      <c r="J53" t="inlineStr">
         <is>
           <t>0x95f0xc45B0x455</t>
         </is>

</xml_diff>